<commit_message>
ACDR2026: one ADRC camera confirmed, set-up from 08:00 per Expo (JM6)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_30_Sep_v2_93.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_30_Sep_v2_93.xlsx
@@ -9680,7 +9680,7 @@
 (3) Gala出発17:30はSC終了16:45の45分後で、撤収要員が不足。
 (4)Day 1全体の前倒しについて、RT・SCは短縮不可のため、日本パビリオン開会式（GOHツアー内）の所要時間次第。　(6)【9/25決定】Day 1前倒しはRTの分割で対応: RT(1) 13:00-15:00、SC 15:15-16:15、RT(2)は29日09:00-09:30（TSは09:30据え置き）。これで17:30のGala出発まで75分の余裕。COSEM（9/29合同会議）と内閣府（9/25 16:30）に提案して確定。SC時の前方席はADRC（所長が説明）と内閣府。事務局席は前方寄り（ADRC席後方）に再配置。
 (5)【9/28内閣府】10/28 16:00-16:30 MHA HQでバイ会談、16:30-16:40 MOC署名式（室長・御手洗参事官）。SC途中で退出、日本側司会は中根補佐。
-(6)【9/29 JM6】名札65枚はSCDF部署から借用（ADRCが国旗ロゴ素材と名簿〈10/13〉を提供）。当日早朝設営の可否をExpoに確認中。AV見積SGD17〜19K、カメラは演台固定1台＋U字パン1台（Sylvia案）、ADRC持込＋職員操作を提案予定。RT(1) 13:00-15:00＝Armenia〜Turkiye 22枠（各5分、Japanの直後に仙台市）、ADRC Opening 12:45-13:00＝Commissioner（tbc）・林副大臣・三浦センター長 各4分。</t>
+(6)【9/29 JM6】名札65枚はSCDF部署から借用（ADRCが国旗ロゴ素材と名簿〈10/13〉を提供）。当日早朝設営の可否をExpoに確認中。AV見積SGD17〜19K。Zoom用カメラ1台はADRC持込で決定、2台運用（演台固定＋U字パン、Sylvia案）は未決。設営開始はExpo最早08:00とSylvia（JM6、要確認）、07:30入室は未承認。RT(1) 13:00-15:00＝Armenia〜Turkiye 22枠（各5分、Japanの直後に仙台市）、ADRC Opening 12:45-13:00＝Commissioner（tbc）・林副大臣・三浦センター長 各4分。</t>
         </is>
       </c>
     </row>
@@ -14853,17 +14853,17 @@
       </c>
       <c r="C55" s="202" t="inlineStr">
         <is>
-          <t>カメラ2台と操作</t>
+          <t>カメラ（Zoom用）の持込と2台運用の可否</t>
         </is>
       </c>
       <c r="D55" s="202" t="inlineStr">
         <is>
-          <t>Sylvia案: 演台固定1台＋U字パン1台（前方中央）。10月はカメラマン確保困難。ADRC: 9/24メールどおり自前カメラ持込＋職員操作（HDMIで業者スイッチャー/Zoom PCへ）を提案。教室型1列目のRT発言者（仙台市・Google）をパンで拾えるか。</t>
+          <t>【決定】Zoom用ビデオカメラ1台はADRCが持込（仙台と同様にHDMI接続、AVオペレータへ渡す）。2台運用（演台固定＋U字パン、Sylvia 9/29案）にするかは未決。10月はカメラマン確保困難、業者機材を職員が操作する場合の損害責任をSylviaが懸念。教室型1列目のRT発言者（仙台市・Google）をどう撮るかも未決。</t>
         </is>
       </c>
       <c r="E55" s="202" t="inlineStr">
         <is>
-          <t>持込の可否、HDMI入力、見積からの減額</t>
+          <t>2台目の要否と費用、HDMI入力、見積からの減額</t>
         </is>
       </c>
       <c r="F55" s="201" t="inlineStr">
@@ -14883,7 +14883,7 @@
       </c>
       <c r="I55" s="203" t="inlineStr">
         <is>
-          <t>未協議</t>
+          <t>協議中</t>
         </is>
       </c>
     </row>
@@ -14952,12 +14952,12 @@
       </c>
       <c r="D57" s="202" t="inlineStr">
         <is>
-          <t>前日設営はExpoが1日分課金。当日早朝の設営可否をSylviaがExpo/COSEMに確認中。</t>
+          <t>前日設営はExpoが1日分課金。JM6でSylvia「Expoに確認したところ設営開始は最早08:00」（録音83:28、要確認）。ADRCの07:30入室希望（9/24メール）は未承認。当日早朝設営の可否と開始時刻をSylviaがExpo/COSEMに確認中。</t>
         </is>
       </c>
       <c r="E57" s="202" t="inlineStr">
         <is>
-          <t>入室可能時刻（07:30）</t>
+          <t>設営開始時刻（08:00か07:30か）、29日はRT(2) 09:00開始のため準備1時間</t>
         </is>
       </c>
       <c r="F57" s="201" t="inlineStr">
@@ -15122,7 +15122,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="B62" s="77" t="inlineStr">
         <is>
@@ -15154,7 +15153,6 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="B67" s="77" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
ACDR2026: same furniture layout both days; 29 Oct morning AV-only set-up
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BHBsW6jxyH2X7L51FtZqxc
</commit_message>
<xml_diff>
--- a/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_30_Sep_v2_93.xlsx
+++ b/reports/acdr2026_staff_deployment/動態表ACDR2026_as_of_30_Sep_v2_93.xlsx
@@ -10014,7 +10014,7 @@
       </c>
       <c r="D4" s="184" t="inlineStr">
         <is>
-          <t>会場準備(ステージ前方へ・テーブルマイク)／登壇者集合・接続確認</t>
+          <t>会場準備（家具は前日のまま。AV・名札のみ）／登壇者集合・接続確認</t>
         </is>
       </c>
       <c r="E4" s="95" t="n"/>
@@ -14952,12 +14952,12 @@
       </c>
       <c r="D57" s="202" t="inlineStr">
         <is>
-          <t>前日設営はExpoが1日分課金。JM6でSylvia「Expoに確認したところ設営開始は最早08:00」（録音83:28、要確認）。ADRCの07:30入室希望（9/24メール）は未承認。当日早朝設営の可否と開始時刻をSylviaがExpo/COSEMに確認中。</t>
+          <t>前日設営はExpoが1日分課金。JM6でSylvia「Expoに確認したところ設営開始は最早08:00」（録音83:28、要確認）。ADRCの07:30入室希望（9/24メール）は未承認。当日早朝設営の可否と開始時刻をSylviaがExpo/COSEMに確認中。【荒木田 9/30】机・椅子の配置を28・29日で共通にし（前方登壇者卓・演台・ステージは28日朝に設営してそのまま）、29日朝はAVと名札の準備のみとすれば08:00入室で足りる。9/24メールの「28日夜の前方組替」は不要。</t>
         </is>
       </c>
       <c r="E57" s="202" t="inlineStr">
         <is>
-          <t>設営開始時刻（08:00か07:30か）、29日はRT(2) 09:00開始のため準備1時間</t>
+          <t>設営開始時刻（08:00）、28日の前方構成を29日と同じにする可否（RT・SCでも登壇者卓を置いたまま）</t>
         </is>
       </c>
       <c r="F57" s="201" t="inlineStr">

</xml_diff>